<commit_message>
Updated Citizen Charter PDF link
</commit_message>
<xml_diff>
--- a/documents/establishment-order/order details.xlsx
+++ b/documents/establishment-order/order details.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <fileVersion appName="Polaris Office Sheet" lastEdited="5" lowestEdited="4" rupBuild="10.115.186.54614"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,12 +14,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$19</definedName>
   </definedNames>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>S.No.</t>
   </si>
@@ -165,62 +165,620 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="19">
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="10"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="11"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FFFF0000"/>
+    </font>
+    <font>
+      <sz val="18.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="3"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FF3F3F76"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FF3F3F3F"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FFFA7D00"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FFFA7D00"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="1"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FF006100"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FF9C0006"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FF9C6500"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color theme="0"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+      <color rgb="FF7F7F7F"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599990"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599990"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599990"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599990"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599990"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599990"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399980"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FFACCCEA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.399980"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="7" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="5" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="0" applyFont="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="8" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="26" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="27" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="30" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="31" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="34" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -240,16 +798,57 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
+    <cellStyle name="20% - Accent1" xfId="25" builtinId="30"/>
+    <cellStyle name="20% - Accent2" xfId="29" builtinId="34"/>
+    <cellStyle name="20% - Accent3" xfId="33" builtinId="38"/>
+    <cellStyle name="20% - Accent4" xfId="37" builtinId="42"/>
+    <cellStyle name="20% - Accent5" xfId="41" builtinId="46"/>
+    <cellStyle name="20% - Accent6" xfId="45" builtinId="50"/>
+    <cellStyle name="40% - Accent1" xfId="26" builtinId="31"/>
+    <cellStyle name="40% - Accent2" xfId="30" builtinId="35"/>
+    <cellStyle name="40% - Accent3" xfId="34" builtinId="39"/>
+    <cellStyle name="40% - Accent4" xfId="38" builtinId="43"/>
+    <cellStyle name="40% - Accent5" xfId="42" builtinId="47"/>
+    <cellStyle name="40% - Accent6" xfId="46" builtinId="51"/>
+    <cellStyle name="60% - Accent1" xfId="27" builtinId="32"/>
+    <cellStyle name="60% - Accent2" xfId="31" builtinId="36"/>
+    <cellStyle name="60% - Accent3" xfId="35" builtinId="40"/>
+    <cellStyle name="60% - Accent4" xfId="39" builtinId="44"/>
+    <cellStyle name="60% - Accent5" xfId="43" builtinId="48"/>
+    <cellStyle name="60% - Accent6" xfId="47" builtinId="52"/>
+    <cellStyle name="Accent1" xfId="24" builtinId="29"/>
+    <cellStyle name="Accent2" xfId="28" builtinId="33"/>
+    <cellStyle name="Accent3" xfId="32" builtinId="37"/>
+    <cellStyle name="Accent4" xfId="36" builtinId="41"/>
+    <cellStyle name="Accent5" xfId="40" builtinId="45"/>
+    <cellStyle name="Accent6" xfId="44" builtinId="49"/>
+    <cellStyle name="Bad" xfId="22" builtinId="27"/>
+    <cellStyle name="Calculation" xfId="17" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="18" builtinId="23"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Comment" xfId="8" builtinId="10"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Currency[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Explanatory Text" xfId="48" builtinId="53"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9" hidden="1"/>
+    <cellStyle name="Good" xfId="21" builtinId="26"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8" hidden="1"/>
+    <cellStyle name="Input" xfId="15" builtinId="20"/>
+    <cellStyle name="Linked Cell" xfId="19" builtinId="24"/>
+    <cellStyle name="Neutral" xfId="23" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Output" xfId="16" builtinId="21"/>
+    <cellStyle name="Percentage" xfId="3" builtinId="5"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Title 1" xfId="11" builtinId="16"/>
+    <cellStyle name="Title 2" xfId="12" builtinId="17"/>
+    <cellStyle name="Title 3" xfId="13" builtinId="18"/>
+    <cellStyle name="Title 4" xfId="14" builtinId="19"/>
+    <cellStyle name="Total" xfId="20" builtinId="25"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -539,17 +1138,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.000000"/>
   <cols>
-    <col min="2" max="2" width="45" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="44.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="63.85546875" style="6" customWidth="1"/>
+    <col min="2" max="2" style="1" width="45.00499998" customWidth="1" outlineLevel="0"/>
+    <col min="3" max="3" width="10.43357168" customWidth="1" outlineLevel="0"/>
+    <col min="4" max="4" width="44.57643018" customWidth="1" outlineLevel="0"/>
+    <col min="5" max="5" style="6" width="63.86214338" customWidth="1" outlineLevel="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -564,7 +1163,7 @@
       </c>
       <c r="E1" s="7"/>
     </row>
-    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="30.000000">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -581,7 +1180,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -598,7 +1197,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="30.000000">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -615,7 +1214,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="30.000000">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -632,7 +1231,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="30.000000">
       <c r="A6" s="8">
         <v>6</v>
       </c>
@@ -649,7 +1248,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="30.000000">
       <c r="A7" s="8">
         <v>7</v>
       </c>
@@ -666,7 +1265,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="30.000000">
       <c r="A8" s="8">
         <v>8</v>
       </c>
@@ -683,7 +1282,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="30.000000">
       <c r="A9" s="8">
         <v>9</v>
       </c>
@@ -700,7 +1299,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="30.000000">
       <c r="A10" s="8">
         <v>10</v>
       </c>
@@ -717,7 +1316,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="A11" s="8">
         <v>11</v>
       </c>
@@ -730,7 +1329,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="30.000000">
       <c r="A12" s="8">
         <v>12</v>
       </c>
@@ -747,7 +1346,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5">
       <c r="A13" s="8">
         <v>13</v>
       </c>
@@ -764,7 +1363,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5">
       <c r="A14" s="8">
         <v>14</v>
       </c>
@@ -781,7 +1380,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="30.000000">
       <c r="A15" s="8">
         <v>15</v>
       </c>
@@ -798,7 +1397,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="30.000000">
       <c r="A16" s="8">
         <v>16</v>
       </c>
@@ -815,7 +1414,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="30.000000">
       <c r="A17" s="8">
         <v>17</v>
       </c>
@@ -832,7 +1431,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="30.000000">
       <c r="A18" s="8">
         <v>18</v>
       </c>
@@ -849,7 +1448,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="30.000000">
       <c r="A19" s="8">
         <v>19</v>
       </c>
@@ -868,29 +1467,34 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D19">
-    <sortState ref="A2:D17">
+    <sortState ref="A2:D19">
       <sortCondition ref="B1:B17"/>
     </sortState>
   </autoFilter>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.000000"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.000000"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>